<commit_message>
Just testing the new authoring process, adjusted test data and tested results.
</commit_message>
<xml_diff>
--- a/rules/CORE-000289/negative/01/data/unit-test-coreid-CG0181-negative.xlsx
+++ b/rules/CORE-000289/negative/01/data/unit-test-coreid-CG0181-negative.xlsx
@@ -67,7 +67,7 @@
     <t>LBORNRHI</t>
   </si>
   <si>
-    <t>NEGATIVE</t>
+    <t>30</t>
   </si>
   <si>
     <t>POSITIVE</t>
@@ -170,6 +170,9 @@
     <t>Albumin</t>
   </si>
   <si>
+    <t>NEGATIVE</t>
+  </si>
+  <si>
     <t>g/L</t>
   </si>
   <si>
@@ -177,9 +180,6 @@
   </si>
   <si>
     <t>3.5</t>
-  </si>
-  <si>
-    <t>30</t>
   </si>
   <si>
     <t>Prot</t>
@@ -521,7 +521,7 @@
       <rgbColor rgb="ffb2b2b2"/>
       <rgbColor rgb="ffffffcc"/>
       <rgbColor rgb="ff9bbb59"/>
-      <rgbColor rgb="fff79646"/>
+      <rgbColor rgb="fffefb00"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -2100,25 +2100,25 @@
         <v>49</v>
       </c>
       <c r="G5" t="s" s="15">
+        <v>50</v>
+      </c>
+      <c r="H5" t="s" s="15">
+        <v>51</v>
+      </c>
+      <c r="I5" t="s" s="15">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s" s="15">
+        <v>52</v>
+      </c>
+      <c r="K5" t="s" s="15">
+        <v>51</v>
+      </c>
+      <c r="L5" t="s" s="16">
+        <v>53</v>
+      </c>
+      <c r="M5" t="s" s="17">
         <v>17</v>
-      </c>
-      <c r="H5" t="s" s="15">
-        <v>50</v>
-      </c>
-      <c r="I5" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="J5" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="K5" t="s" s="15">
-        <v>50</v>
-      </c>
-      <c r="L5" t="s" s="16">
-        <v>52</v>
-      </c>
-      <c r="M5" t="s" s="17">
-        <v>53</v>
       </c>
     </row>
     <row r="6" ht="39.55" customHeight="1">
@@ -2183,22 +2183,22 @@
       </c>
       <c r="G7" s="15"/>
       <c r="H7" t="s" s="15">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I7" t="s" s="15">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s" s="15">
+        <v>52</v>
+      </c>
+      <c r="K7" t="s" s="15">
         <v>51</v>
       </c>
-      <c r="J7" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="K7" t="s" s="15">
-        <v>50</v>
-      </c>
       <c r="L7" t="s" s="16">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s" s="22">
-        <v>53</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" ht="39.55" customHeight="1">

</xml_diff>

<commit_message>
Edited rule as per latest decision, pending confirmation on treatment of amount of spaces allowed. Also edited test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000289/negative/01/data/unit-test-coreid-CG0181-negative.xlsx
+++ b/rules/CORE-000289/negative/01/data/unit-test-coreid-CG0181-negative.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="68">
   <si>
     <t>Product</t>
   </si>
@@ -58,21 +58,45 @@
     <t>Error value</t>
   </si>
   <si>
-    <t>Lb.xpt</t>
-  </si>
-  <si>
     <t>Record</t>
   </si>
   <si>
+    <t>LBORRES</t>
+  </si>
+  <si>
+    <t>NEGATIVE</t>
+  </si>
+  <si>
     <t>LBORNRHI</t>
   </si>
   <si>
     <t>30</t>
   </si>
   <si>
+    <t>LBTESTCD</t>
+  </si>
+  <si>
+    <t>ALB</t>
+  </si>
+  <si>
     <t>POSITIVE</t>
   </si>
   <si>
+    <t>ALP</t>
+  </si>
+  <si>
+    <t>&lt; + 30</t>
+  </si>
+  <si>
+    <t>+30</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - &gt; 35.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -35.55</t>
+  </si>
+  <si>
     <t>STUDYID</t>
   </si>
   <si>
@@ -85,13 +109,7 @@
     <t>LBSEQ</t>
   </si>
   <si>
-    <t>LBTESTCD</t>
-  </si>
-  <si>
     <t>LBTEST</t>
-  </si>
-  <si>
-    <t>LBORRES</t>
   </si>
   <si>
     <t>LBORRESU</t>
@@ -161,7 +179,7 @@
     <t>LB</t>
   </si>
   <si>
-    <t>ALB</t>
+    <t>Xyz01</t>
   </si>
   <si>
     <t>1</t>
@@ -170,9 +188,6 @@
     <t>Albumin</t>
   </si>
   <si>
-    <t>NEGATIVE</t>
-  </si>
-  <si>
     <t>g/L</t>
   </si>
   <si>
@@ -182,15 +197,9 @@
     <t>3.5</t>
   </si>
   <si>
-    <t>Prot</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
-    <t>ALP</t>
-  </si>
-  <si>
     <t>Alkaline Phosphatase</t>
   </si>
   <si>
@@ -206,7 +215,13 @@
     <t>3</t>
   </si>
   <si>
-    <t>24</t>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
 </sst>
 </file>
@@ -271,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -311,6 +326,36 @@
     </border>
     <border>
       <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="11"/>
       </left>
       <right style="thin">
@@ -336,21 +381,6 @@
       </top>
       <bottom style="thin">
         <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -401,10 +431,62 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="13"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
         <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="10"/>
       </right>
       <top style="thin">
         <color indexed="13"/>
@@ -420,7 +502,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -442,61 +524,94 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1590,7 +1705,7 @@
     <col min="6" max="16384" width="8.85156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
@@ -1601,7 +1716,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" ht="13.55" customHeight="1">
+    <row r="2" ht="13.5" customHeight="1">
       <c r="A2" t="s" s="4">
         <v>2</v>
       </c>
@@ -1612,56 +1727,56 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
+    <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" ht="13.55" customHeight="1">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" ht="13.55" customHeight="1">
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" ht="13.55" customHeight="1">
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" ht="13.55" customHeight="1">
+    <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" ht="13.55" customHeight="1">
+    <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" ht="13.55" customHeight="1">
+    <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -1686,7 +1801,7 @@
     <col min="6" max="16384" width="8.85156" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>4</v>
       </c>
@@ -1697,7 +1812,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" ht="13.55" customHeight="1">
+    <row r="2" ht="13.5" customHeight="1">
       <c r="A2" t="s" s="4">
         <v>6</v>
       </c>
@@ -1708,56 +1823,56 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
+    <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" ht="13.55" customHeight="1">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" ht="13.55" customHeight="1">
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" ht="13.55" customHeight="1">
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" ht="13.55" customHeight="1">
+    <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" ht="13.55" customHeight="1">
+    <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" ht="13.55" customHeight="1">
+    <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -1775,14 +1890,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="6" width="8.85156" style="6" customWidth="1"/>
     <col min="7" max="16384" width="8.85156" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>8</v>
       </c>
@@ -1798,105 +1913,369 @@
       <c r="E1" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="F1" t="s" s="2">
+      <c r="F1" t="s" s="7">
         <v>13</v>
       </c>
     </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="7">
+    <row r="2" ht="13.5" customHeight="1">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
       <c r="B2" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="C2" t="s" s="4">
+      <c r="D2" s="8">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s" s="9">
         <v>15</v>
       </c>
-      <c r="D2" s="7">
+      <c r="F2" t="s" s="10">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D3" s="8">
         <v>5</v>
       </c>
-      <c r="E2" t="s" s="4">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s" s="4">
+      <c r="E3" t="s" s="11">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="7">
+      <c r="F3" t="s" s="12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" ht="13.5" customHeight="1">
+      <c r="A4" s="8">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D4" s="8">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s" s="9">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s" s="10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" ht="13.5" customHeight="1">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="4">
+      <c r="B5" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="C3" t="s" s="4">
+      <c r="D5" s="8">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s" s="13">
         <v>15</v>
       </c>
-      <c r="D3" s="7">
+      <c r="F5" t="s" s="13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="13.55" customHeight="1">
+      <c r="A6" s="8">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s" s="4">
         <v>6</v>
       </c>
-      <c r="E3" t="s" s="4">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s" s="4">
+      <c r="C6" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D6" s="8">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s" s="4">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s" s="14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" ht="13.5" customHeight="1">
+      <c r="A7" s="8">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D7" s="8">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s" s="15">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s" s="12">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" ht="13.55" customHeight="1">
+      <c r="A8" s="8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D8" s="8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s" s="10">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" ht="13.55" customHeight="1">
+      <c r="A9" s="8">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D9" s="8">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s" s="11">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s" s="12">
         <v>18</v>
       </c>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
+      <c r="A10" s="8">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D10" s="8">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s" s="9">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s" s="10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" ht="13.55" customHeight="1">
+      <c r="A11" s="8">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D11" s="8">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s" s="13">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s" s="10">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" ht="13.55" customHeight="1">
+      <c r="A12" s="8">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D12" s="8">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s" s="4">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s" s="12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" ht="13.55" customHeight="1">
+      <c r="A13" s="8">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D13" s="8">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s" s="15">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s" s="12">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" ht="13.55" customHeight="1">
+      <c r="A14" s="8">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D14" s="8">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s" s="13">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" ht="13.55" customHeight="1">
+      <c r="A15" s="8">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D15" s="8">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s" s="11">
+        <v>17</v>
+      </c>
+      <c r="F15" t="s" s="14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" ht="13.55" customHeight="1">
+      <c r="A16" s="8">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D16" s="8">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s" s="9">
+        <v>19</v>
+      </c>
+      <c r="F16" t="s" s="10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" ht="13.55" customHeight="1">
+      <c r="A17" s="8">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D17" s="8">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s" s="13">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s" s="13">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" ht="13.55" customHeight="1">
+      <c r="A18" s="8">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D18" s="8">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s" s="4">
+        <v>17</v>
+      </c>
+      <c r="F18" t="s" s="14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" ht="13.55" customHeight="1">
+      <c r="A19" s="8">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D19" s="8">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s" s="9">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s" s="11">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1909,366 +2288,437 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="13" width="8.85156" style="8" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="8" customWidth="1"/>
+    <col min="1" max="13" width="8.85156" style="16" customWidth="1"/>
+    <col min="14" max="16384" width="8.85156" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.55" customHeight="1">
-      <c r="A1" t="s" s="9">
+    <row r="1" ht="26.65" customHeight="1">
+      <c r="A1" t="s" s="17">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s" s="17">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s" s="17">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s" s="17">
+        <v>30</v>
+      </c>
+      <c r="E1" t="s" s="17">
         <v>19</v>
       </c>
-      <c r="B1" t="s" s="9">
+      <c r="F1" t="s" s="17">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s" s="17">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s" s="17">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s" s="17">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s" s="17">
+        <v>34</v>
+      </c>
+      <c r="K1" t="s" s="17">
+        <v>35</v>
+      </c>
+      <c r="L1" t="s" s="17">
+        <v>36</v>
+      </c>
+      <c r="M1" t="s" s="17">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" ht="78.6" customHeight="1">
+      <c r="A2" t="s" s="18">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s" s="18">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s" s="18">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s" s="18">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s" s="18">
+        <v>41</v>
+      </c>
+      <c r="F2" t="s" s="18">
+        <v>42</v>
+      </c>
+      <c r="G2" t="s" s="18">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s" s="18">
+        <v>44</v>
+      </c>
+      <c r="I2" t="s" s="18">
+        <v>45</v>
+      </c>
+      <c r="J2" t="s" s="18">
+        <v>46</v>
+      </c>
+      <c r="K2" t="s" s="18">
+        <v>47</v>
+      </c>
+      <c r="L2" t="s" s="18">
+        <v>48</v>
+      </c>
+      <c r="M2" t="s" s="18">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="A3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="C3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s" s="18">
+        <v>51</v>
+      </c>
+      <c r="E3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="I3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="J3" t="s" s="18">
+        <v>51</v>
+      </c>
+      <c r="K3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="L3" t="s" s="18">
+        <v>50</v>
+      </c>
+      <c r="M3" t="s" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" ht="13.5" customHeight="1">
+      <c r="A4" s="19">
+        <v>50</v>
+      </c>
+      <c r="B4" s="19">
+        <v>50</v>
+      </c>
+      <c r="C4" s="19">
+        <v>50</v>
+      </c>
+      <c r="D4" s="19">
+        <v>8</v>
+      </c>
+      <c r="E4" s="19">
+        <v>50</v>
+      </c>
+      <c r="F4" s="19">
+        <v>50</v>
+      </c>
+      <c r="G4" s="19">
+        <v>50</v>
+      </c>
+      <c r="H4" s="19">
+        <v>50</v>
+      </c>
+      <c r="I4" s="19">
+        <v>50</v>
+      </c>
+      <c r="J4" s="19">
+        <v>8</v>
+      </c>
+      <c r="K4" s="19">
+        <v>50</v>
+      </c>
+      <c r="L4" s="19">
+        <v>50</v>
+      </c>
+      <c r="M4" s="20">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" ht="13.5" customHeight="1">
+      <c r="A5" s="21">
+        <v>123101</v>
+      </c>
+      <c r="B5" t="s" s="11">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s" s="13">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s" s="22">
         <v>20</v>
       </c>
-      <c r="C1" t="s" s="9">
+      <c r="F5" t="s" s="13">
+        <v>55</v>
+      </c>
+      <c r="G5" t="s" s="22">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s" s="13">
+        <v>56</v>
+      </c>
+      <c r="I5" t="s" s="13">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s" s="13">
+        <v>57</v>
+      </c>
+      <c r="K5" t="s" s="13">
+        <v>56</v>
+      </c>
+      <c r="L5" t="s" s="23">
+        <v>58</v>
+      </c>
+      <c r="M5" t="s" s="24">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" ht="39.6" customHeight="1">
+      <c r="A6" s="25">
+        <v>123101</v>
+      </c>
+      <c r="B6" t="s" s="14">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s" s="9">
+        <v>59</v>
+      </c>
+      <c r="E6" t="s" s="26">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s" s="9">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s" s="26">
         <v>21</v>
       </c>
-      <c r="D1" t="s" s="9">
+      <c r="H6" t="s" s="9">
+        <v>61</v>
+      </c>
+      <c r="I6" t="s" s="9">
+        <v>62</v>
+      </c>
+      <c r="J6" t="s" s="9">
+        <v>62</v>
+      </c>
+      <c r="K6" t="s" s="9">
+        <v>61</v>
+      </c>
+      <c r="L6" t="s" s="27">
+        <v>63</v>
+      </c>
+      <c r="M6" t="s" s="24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" ht="13.55" customHeight="1">
+      <c r="A7" s="28">
+        <v>123101</v>
+      </c>
+      <c r="B7" t="s" s="12">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s" s="10">
+        <v>64</v>
+      </c>
+      <c r="E7" t="s" s="29">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s" s="10">
+        <v>55</v>
+      </c>
+      <c r="G7" t="s" s="29">
+        <v>23</v>
+      </c>
+      <c r="H7" t="s" s="10">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s" s="10">
+        <v>57</v>
+      </c>
+      <c r="J7" t="s" s="10">
+        <v>57</v>
+      </c>
+      <c r="K7" t="s" s="10">
+        <v>56</v>
+      </c>
+      <c r="L7" t="s" s="30">
+        <v>58</v>
+      </c>
+      <c r="M7" t="s" s="24">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" ht="13.55" customHeight="1">
+      <c r="A8" s="21">
+        <v>123101</v>
+      </c>
+      <c r="B8" t="s" s="11">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s" s="13">
+        <v>65</v>
+      </c>
+      <c r="E8" t="s" s="22">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s" s="13">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s" s="22">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s" s="13">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s" s="13">
+        <v>57</v>
+      </c>
+      <c r="J8" t="s" s="13">
+        <v>57</v>
+      </c>
+      <c r="K8" t="s" s="13">
+        <v>56</v>
+      </c>
+      <c r="L8" t="s" s="23">
+        <v>58</v>
+      </c>
+      <c r="M8" t="s" s="24">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" ht="13.55" customHeight="1">
+      <c r="A9" s="31">
+        <v>123101</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s" s="15">
+        <v>66</v>
+      </c>
+      <c r="E9" t="s" s="32">
         <v>22</v>
       </c>
-      <c r="E1" t="s" s="9">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s" s="9">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s" s="9">
+      <c r="F9" t="s" s="15">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s" s="32">
         <v>25</v>
       </c>
-      <c r="H1" t="s" s="9">
+      <c r="H9" t="s" s="15">
+        <v>61</v>
+      </c>
+      <c r="I9" t="s" s="15">
+        <v>62</v>
+      </c>
+      <c r="J9" t="s" s="15">
+        <v>62</v>
+      </c>
+      <c r="K9" t="s" s="15">
+        <v>61</v>
+      </c>
+      <c r="L9" t="s" s="33">
+        <v>63</v>
+      </c>
+      <c r="M9" t="s" s="24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" ht="13.55" customHeight="1">
+      <c r="A10" s="25">
+        <v>123101</v>
+      </c>
+      <c r="B10" t="s" s="14">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s" s="10">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s" s="9">
+        <v>67</v>
+      </c>
+      <c r="E10" t="s" s="26">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s" s="9">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s" s="26">
         <v>26</v>
       </c>
-      <c r="I1" t="s" s="9">
-        <v>27</v>
-      </c>
-      <c r="J1" t="s" s="9">
-        <v>28</v>
-      </c>
-      <c r="K1" t="s" s="9">
-        <v>29</v>
-      </c>
-      <c r="L1" t="s" s="9">
-        <v>30</v>
-      </c>
-      <c r="M1" t="s" s="9">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" ht="78.55" customHeight="1">
-      <c r="A2" t="s" s="10">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s" s="10">
-        <v>33</v>
-      </c>
-      <c r="D2" t="s" s="10">
-        <v>34</v>
-      </c>
-      <c r="E2" t="s" s="10">
-        <v>35</v>
-      </c>
-      <c r="F2" t="s" s="10">
-        <v>36</v>
-      </c>
-      <c r="G2" t="s" s="10">
-        <v>37</v>
-      </c>
-      <c r="H2" t="s" s="10">
-        <v>38</v>
-      </c>
-      <c r="I2" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="J2" t="s" s="10">
-        <v>40</v>
-      </c>
-      <c r="K2" t="s" s="10">
-        <v>41</v>
-      </c>
-      <c r="L2" t="s" s="10">
-        <v>42</v>
-      </c>
-      <c r="M2" t="s" s="10">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="B3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="C3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s" s="10">
-        <v>45</v>
-      </c>
-      <c r="E3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="F3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="G3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="H3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="I3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="J3" t="s" s="10">
-        <v>45</v>
-      </c>
-      <c r="K3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="L3" t="s" s="10">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s" s="10">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="11">
-        <v>50</v>
-      </c>
-      <c r="B4" s="11">
-        <v>50</v>
-      </c>
-      <c r="C4" s="11">
-        <v>50</v>
-      </c>
-      <c r="D4" s="11">
-        <v>8</v>
-      </c>
-      <c r="E4" s="11">
-        <v>50</v>
-      </c>
-      <c r="F4" s="11">
-        <v>50</v>
-      </c>
-      <c r="G4" s="11">
-        <v>50</v>
-      </c>
-      <c r="H4" s="11">
-        <v>50</v>
-      </c>
-      <c r="I4" s="11">
-        <v>50</v>
-      </c>
-      <c r="J4" s="11">
-        <v>8</v>
-      </c>
-      <c r="K4" s="11">
-        <v>50</v>
-      </c>
-      <c r="L4" s="11">
-        <v>50</v>
-      </c>
-      <c r="M4" s="12">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="13">
-        <v>123101</v>
-      </c>
-      <c r="B5" t="s" s="14">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s" s="15">
-        <v>47</v>
-      </c>
-      <c r="D5" t="s" s="15">
-        <v>48</v>
-      </c>
-      <c r="E5" t="s" s="15">
-        <v>47</v>
-      </c>
-      <c r="F5" t="s" s="15">
-        <v>49</v>
-      </c>
-      <c r="G5" t="s" s="15">
-        <v>50</v>
-      </c>
-      <c r="H5" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="I5" t="s" s="15">
-        <v>52</v>
-      </c>
-      <c r="J5" t="s" s="15">
-        <v>52</v>
-      </c>
-      <c r="K5" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="L5" t="s" s="16">
-        <v>53</v>
-      </c>
-      <c r="M5" t="s" s="17">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" ht="39.55" customHeight="1">
-      <c r="A6" s="18">
-        <v>123101</v>
-      </c>
-      <c r="B6" t="s" s="19">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s" s="20">
-        <v>54</v>
-      </c>
-      <c r="D6" t="s" s="20">
-        <v>55</v>
-      </c>
-      <c r="E6" t="s" s="20">
-        <v>56</v>
-      </c>
-      <c r="F6" t="s" s="20">
-        <v>57</v>
-      </c>
-      <c r="G6" t="s" s="20">
-        <v>18</v>
-      </c>
-      <c r="H6" t="s" s="20">
-        <v>58</v>
-      </c>
-      <c r="I6" t="s" s="20">
-        <v>59</v>
-      </c>
-      <c r="J6" t="s" s="20">
-        <v>59</v>
-      </c>
-      <c r="K6" t="s" s="20">
-        <v>58</v>
-      </c>
-      <c r="L6" t="s" s="21">
-        <v>60</v>
-      </c>
-      <c r="M6" t="s" s="17">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="13">
-        <v>123101</v>
-      </c>
-      <c r="B7" t="s" s="14">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s" s="15">
-        <v>47</v>
-      </c>
-      <c r="D7" t="s" s="15">
+      <c r="H10" t="s" s="9">
         <v>61</v>
       </c>
-      <c r="E7" t="s" s="15">
-        <v>47</v>
-      </c>
-      <c r="F7" t="s" s="15">
-        <v>49</v>
-      </c>
-      <c r="G7" s="15"/>
-      <c r="H7" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="I7" t="s" s="15">
-        <v>52</v>
-      </c>
-      <c r="J7" t="s" s="15">
-        <v>52</v>
-      </c>
-      <c r="K7" t="s" s="15">
-        <v>51</v>
-      </c>
-      <c r="L7" t="s" s="16">
-        <v>53</v>
-      </c>
-      <c r="M7" t="s" s="22">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" ht="39.55" customHeight="1">
-      <c r="A8" s="23">
-        <v>123101</v>
-      </c>
-      <c r="B8" t="s" s="4">
-        <v>46</v>
-      </c>
-      <c r="C8" t="s" s="24">
-        <v>54</v>
-      </c>
-      <c r="D8" t="s" s="24">
+      <c r="I10" t="s" s="9">
         <v>62</v>
       </c>
-      <c r="E8" t="s" s="24">
-        <v>56</v>
-      </c>
-      <c r="F8" t="s" s="24">
-        <v>57</v>
-      </c>
-      <c r="G8" s="24"/>
-      <c r="H8" t="s" s="24">
-        <v>58</v>
-      </c>
-      <c r="I8" t="s" s="24">
-        <v>59</v>
-      </c>
-      <c r="J8" t="s" s="24">
-        <v>59</v>
-      </c>
-      <c r="K8" t="s" s="24">
-        <v>58</v>
-      </c>
-      <c r="L8" t="s" s="24">
-        <v>60</v>
-      </c>
-      <c r="M8" t="s" s="20">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="25"/>
-    </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
+      <c r="J10" t="s" s="9">
+        <v>62</v>
+      </c>
+      <c r="K10" t="s" s="9">
+        <v>61</v>
+      </c>
+      <c r="L10" t="s" s="27">
+        <v>63</v>
+      </c>
+      <c r="M10" t="s" s="24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" ht="13.55" customHeight="1">
+      <c r="A11" s="34"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="35"/>
+      <c r="K11" s="35"/>
+      <c r="L11" s="35"/>
+      <c r="M11" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>